<commit_message>
Update device control documents and editable diagrams
</commit_message>
<xml_diff>
--- a/artifacts/reports/device-control/40_プログラム仕様書/デバイスコネクタ/プログラム仕様書_端末アプリ_デバイスコネクタ_カスタマディスプレイ制御_SHARP/プログラム仕様書_端末アプリ_デバイスコネクタ_カスタマディスプレイ制御_SHARP_Ver0.1.1.xlsx
+++ b/artifacts/reports/device-control/40_プログラム仕様書/デバイスコネクタ/プログラム仕様書_端末アプリ_デバイスコネクタ_カスタマディスプレイ制御_SHARP/プログラム仕様書_端末アプリ_デバイスコネクタ_カスタマディスプレイ制御_SHARP_Ver0.1.1.xlsx
@@ -21,11 +21,10 @@
   <numFmts count="0"/>
   <fonts count="8">
     <font>
-      <name val="Calibri"/>
+      <name val="Meiryo UI"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
@@ -953,9 +952,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Meiryo UI"/>
+        <a:ea typeface="Meiryo UI"/>
+        <a:cs typeface="Meiryo UI"/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
@@ -987,9 +986,9 @@
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Meiryo UI"/>
+        <a:ea typeface="Meiryo UI"/>
+        <a:cs typeface="Meiryo UI"/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>

</xml_diff>